<commit_message>
Add_Soundfx + Menu Music
</commit_message>
<xml_diff>
--- a/Signomaly/GDD/Signomaly.xlsx
+++ b/Signomaly/GDD/Signomaly.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\Unity_GameMaking\0. Projects\170426_LD_GameJam59\LD59_Signomaly\Signomaly\GDD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C8295F0-FEA2-49DE-A960-DDA1415338B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3610BDF7-BEDE-4B5D-9500-2F7820256ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{93CE968A-0C34-467A-AF09-AD4AE7C1ADD9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{93CE968A-0C34-467A-AF09-AD4AE7C1ADD9}"/>
   </bookViews>
   <sheets>
     <sheet name="Gameplay_Overview" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="306">
   <si>
     <t>SIGNOMALY</t>
   </si>
@@ -2611,6 +2611,9 @@
   </si>
   <si>
     <t>Sẵn sàng</t>
+  </si>
+  <si>
+    <t>Add vào Menu. Không có nhạc in-game</t>
   </si>
 </sst>
 </file>
@@ -9442,6 +9445,11 @@
         <v>285</v>
       </c>
     </row>
+    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>305</v>
+      </c>
+    </row>
     <row r="17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>